<commit_message>
Clean featured artist titles
</commit_message>
<xml_diff>
--- a/reports/site-audit/2026-07-10/icerik-denetim-2026-07-10.xlsx
+++ b/reports/site-audit/2026-07-10/icerik-denetim-2026-07-10.xlsx
@@ -442,8 +442,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
@@ -963,17 +963,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The Weeknd</t>
+          <t>The Weeknd, Lana Del Rey</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The Abyss Türkçe Çeviri (ft. Lana Del Rey)</t>
+          <t>The Abyss</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The Weeknd The Abyss Türkçe Çeviri (ft. Lana Del Rey)</t>
+          <t>The Weeknd, Lana Del Rey The Abyss Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1005,17 +1005,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The Weeknd</t>
+          <t>The Weeknd, Future</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enjoy The Show Türkçe Çeviri (ft. Future)</t>
+          <t>Enjoy The Show</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>The Weeknd Enjoy The Show Türkçe Çeviri (ft. Future)</t>
+          <t>The Weeknd, Future Enjoy The Show Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1047,17 +1047,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>The Weeknd</t>
+          <t>The Weeknd, Travis Scott</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Reflections Laughing Türkçe Çeviri (ft. Travis Scott)</t>
+          <t>Reflections Laughing</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>The Weeknd Reflections Laughing Türkçe Çeviri (ft. Travis Scott)</t>
+          <t>The Weeknd, Travis Scott Reflections Laughing Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1598,12 +1598,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ENHYPEN Paul Russell Confessions</t>
+          <t>ENHYPEN Paul Russell Confessions</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Flo Rida ENHYPEN Paul Russell Confessions Türkçe Çeviri</t>
+          <t>Flo Rida ENHYPEN Paul Russell Confessions Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3572,12 +3572,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve"> That's So True</t>
+          <t>That's So True</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Gracie Abrams That's So True Türkçe Çeviri</t>
+          <t>Gracie Abrams That's So True Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -4407,17 +4407,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>KATSEYE</t>
+          <t>KATSEYE, YEONJUN</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>ft Yeonjun Touch</t>
+          <t>Touch</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>KATSEYE ft Yeonjun Touch Türkçe Çeviri</t>
+          <t>KATSEYE, YEONJUN Touch Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -5583,17 +5583,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Katy Perry</t>
+          <t>Katy Perry, Doechii</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Doechii I'M HIS, HE'S MINE</t>
+          <t>I'M HIS, HE'S MINE</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Katy Perry Doechii I'M HIS, HE'S MINE </t>
+          <t>Katy Perry, Doechii I'M HIS, HE'S MINE Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5835,12 +5835,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Hello, World</t>
+          <t>BAEKHYUN</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>BAEKHYUN Pineapple Slice</t>
+          <t>Pineapple Slice</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -6591,17 +6591,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>B.I</t>
+          <t>B.I, Soulja Boy, DeVita</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>BI Soulja Boy BTBT ft DeVita</t>
+          <t>BTBT</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>BI Soulja Boy BTBT ft DeVita Türkçe Çeviri</t>
+          <t>B.I, Soulja Boy, DeVita BTBT Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -7767,17 +7767,17 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Lady Gaga</t>
+          <t>Lady Gaga, Bruno Mars</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Bruno Mars Die With A Smile</t>
+          <t>Die With A Smile</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Lady Gaga Bruno Mars Die With A Smile Türkçe Çeviri</t>
+          <t>Lady Gaga, Bruno Mars Die With A Smile Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -8108,12 +8108,12 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>KARINA UP Türkçe Çeviri (Yayınlanmamış Şarkı)</t>
+          <t>KARINA UP (Yayınlanmamış Şarkı)</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>KARINA UP Türkçe Çeviri (Yayınlanmamış Şarkı)</t>
+          <t>Aespa KARINA UP (Yayınlanmamış Şarkı) Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -8397,17 +8397,17 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Charli XCX</t>
+          <t>Charli XCX, Billie Eilish</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>ft Billie Eilish Guess</t>
+          <t>Guess</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Charli XCX ft Billie Eilish Guess Türkçe Çeviri</t>
+          <t>Charli XCX, Billie Eilish Guess Türkçe Çeviri</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">

</xml_diff>